<commit_message>
phase 1: clean-state re-verification, live read-only evidence, verification matrix
Regenerated outputs/ from scratch; reran unit, golden, mutation, grader, pipelines.
Fixes: stale review packet, UI test order dependency, scan_secrets ignoring file
paths, qbo_test_connection exit code on failure (+QBO_MCP_SERVER_DIR override),
loader --apply side effect before env check (found by independent reviewer).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/ABC_Inc_Financial_Analysis.xlsx
+++ b/outputs/ABC_Inc_Financial_Analysis.xlsx
@@ -2526,7 +2526,7 @@
         <v>39.02000000000044</v>
       </c>
       <c r="E73" t="n">
-        <v>0.003121600000000058</v>
+        <v>0.003121600000000035</v>
       </c>
     </row>
     <row r="74">
@@ -2600,7 +2600,7 @@
         <v>-21000</v>
       </c>
       <c r="E77" t="n">
-        <v>-0.8852978584644804</v>
+        <v>-0.8852978584644803</v>
       </c>
     </row>
     <row r="78">
@@ -2657,7 +2657,7 @@
         <v>42.37999999999988</v>
       </c>
       <c r="E80" t="n">
-        <v>0.02975768342262497</v>
+        <v>0.02975768342262502</v>
       </c>
     </row>
     <row r="81">
@@ -2788,7 +2788,7 @@
         <v>-872.7299999999996</v>
       </c>
       <c r="E87" t="n">
-        <v>-0.04565822329854807</v>
+        <v>-0.04565822329854804</v>
       </c>
     </row>
     <row r="88">
@@ -2824,7 +2824,7 @@
         <v>-3137.08</v>
       </c>
       <c r="E89" t="n">
-        <v>-0.4799414966694102</v>
+        <v>-0.4799414966694103</v>
       </c>
     </row>
     <row r="90">
@@ -2843,7 +2843,7 @@
         <v>-13.55000000000001</v>
       </c>
       <c r="E90" t="n">
-        <v>-0.03340729783037477</v>
+        <v>-0.03340729783037478</v>
       </c>
     </row>
     <row r="91">
@@ -2862,7 +2862,7 @@
         <v>1464.460000000001</v>
       </c>
       <c r="E91" t="n">
-        <v>-0.0940201668975772</v>
+        <v>0.09402016689757724</v>
       </c>
     </row>
     <row r="92">
@@ -2881,7 +2881,7 @@
         <v>-262.6199999999999</v>
       </c>
       <c r="E92" t="n">
-        <v>-0.0935049953357876</v>
+        <v>-0.09350499533578764</v>
       </c>
     </row>
     <row r="93">
@@ -2900,7 +2900,7 @@
         <v>738.630000000001</v>
       </c>
       <c r="E93" t="n">
-        <v>0.0284877023051886</v>
+        <v>0.02848770230518867</v>
       </c>
     </row>
     <row r="94">
@@ -2995,7 +2995,7 @@
         <v>-24287.5</v>
       </c>
       <c r="E98" t="n">
-        <v>-0.3966925275622704</v>
+        <v>-0.3966925275622703</v>
       </c>
     </row>
     <row r="99">
@@ -3014,7 +3014,7 @@
         <v>117.8900000000003</v>
       </c>
       <c r="E99" t="n">
-        <v>0.01440469004684664</v>
+        <v>0.01440469004684674</v>
       </c>
     </row>
     <row r="100">
@@ -3033,7 +3033,7 @@
         <v>657.63</v>
       </c>
       <c r="E100" t="n">
-        <v>0.8858520683756079</v>
+        <v>0.8858520683756078</v>
       </c>
     </row>
     <row r="101">
@@ -3052,7 +3052,7 @@
         <v>4.4699999999998</v>
       </c>
       <c r="E101" t="n">
-        <v>0.001157191674433067</v>
+        <v>0.001157191674433002</v>
       </c>
     </row>
     <row r="102">
@@ -3200,7 +3200,7 @@
         <v>-344.9700000000012</v>
       </c>
       <c r="E109" t="n">
-        <v>-0.01105747147805736</v>
+        <v>-0.01105747147805738</v>
       </c>
     </row>
     <row r="110">
@@ -3219,7 +3219,7 @@
         <v>645.6300000000001</v>
       </c>
       <c r="E110" t="n">
-        <v>0.7884979421355383</v>
+        <v>0.7884979421355384</v>
       </c>
     </row>
     <row r="111">
@@ -3257,7 +3257,7 @@
         <v>-149.1800000000003</v>
       </c>
       <c r="E112" t="n">
-        <v>-0.06310250455777922</v>
+        <v>-0.06310250455777923</v>
       </c>
     </row>
     <row r="113">
@@ -3295,7 +3295,7 @@
         <v>-49</v>
       </c>
       <c r="E114" t="n">
-        <v>-0.03450995858804973</v>
+        <v>-0.03450995858804969</v>
       </c>
     </row>
     <row r="115">
@@ -3314,7 +3314,7 @@
         <v>334.86</v>
       </c>
       <c r="E115" t="n">
-        <v>0.6681298509547278</v>
+        <v>0.6681298509547277</v>
       </c>
     </row>
     <row r="116">
@@ -3350,7 +3350,7 @@
         <v>2460.19</v>
       </c>
       <c r="E117" t="n">
-        <v>35.94141709276844</v>
+        <v>35.94141709276845</v>
       </c>
     </row>
     <row r="118">
@@ -3405,7 +3405,7 @@
         <v>736.6800000000003</v>
       </c>
       <c r="E120" t="n">
-        <v>0.3090865608518889</v>
+        <v>0.3090865608518888</v>
       </c>
     </row>
     <row r="121">
@@ -3536,7 +3536,7 @@
         <v>1136.96</v>
       </c>
       <c r="E127" t="n">
-        <v>0.3309156528319459</v>
+        <v>0.330915652831946</v>
       </c>
     </row>
     <row r="128">
@@ -3606,7 +3606,7 @@
         <v>17906.97</v>
       </c>
       <c r="E131" t="n">
-        <v>0.2400630141331355</v>
+        <v>0.2400630141331354</v>
       </c>
     </row>
     <row r="132">
@@ -3625,7 +3625,7 @@
         <v>525.5200000000004</v>
       </c>
       <c r="E132" t="n">
-        <v>0.06366258539002301</v>
+        <v>0.06366258539002304</v>
       </c>
     </row>
     <row r="133">
@@ -3644,7 +3644,7 @@
         <v>1709.89</v>
       </c>
       <c r="E133" t="n">
-        <v>0.8159234605015149</v>
+        <v>0.815923460501515</v>
       </c>
     </row>
     <row r="134">
@@ -3716,7 +3716,7 @@
         <v>7119.699999999999</v>
       </c>
       <c r="E137" t="n">
-        <v>0.5395248949700824</v>
+        <v>0.5395248949700823</v>
       </c>
     </row>
     <row r="138">
@@ -3771,7 +3771,7 @@
         <v>-836.0699999999997</v>
       </c>
       <c r="E140" t="n">
-        <v>-0.05117340087330258</v>
+        <v>-0.05117340087330256</v>
       </c>
     </row>
     <row r="141">
@@ -3824,7 +3824,7 @@
         <v>-30.02000000000044</v>
       </c>
       <c r="E143" t="n">
-        <v>-0.002394126494734028</v>
+        <v>-0.002394126494734073</v>
       </c>
     </row>
     <row r="144">
@@ -3949,7 +3949,7 @@
         <v>43.54999999999995</v>
       </c>
       <c r="E150" t="n">
-        <v>0.02969554396372431</v>
+        <v>0.02969554396372436</v>
       </c>
     </row>
     <row r="151">
@@ -4004,7 +4004,7 @@
         <v>47.06999999999999</v>
       </c>
       <c r="E153" t="n">
-        <v>0.1286944634313054</v>
+        <v>0.1286944634313055</v>
       </c>
     </row>
     <row r="154">
@@ -4133,7 +4133,7 @@
         <v>100.02</v>
       </c>
       <c r="E160" t="n">
-        <v>0.255120520341793</v>
+        <v>0.2551205203417931</v>
       </c>
     </row>
     <row r="161">
@@ -4152,7 +4152,7 @@
         <v>-1555</v>
       </c>
       <c r="E161" t="n">
-        <v>0.110193345030599</v>
+        <v>-0.110193345030599</v>
       </c>
     </row>
     <row r="162">
@@ -4228,7 +4228,7 @@
         <v>-507.27</v>
       </c>
       <c r="E165" t="n">
-        <v>-0.5117529558936282</v>
+        <v>-0.5117529558936281</v>
       </c>
     </row>
     <row r="166">
@@ -4304,7 +4304,7 @@
         <v>67.52999999999884</v>
       </c>
       <c r="E169" t="n">
-        <v>0.008134155140369081</v>
+        <v>0.008134155140369142</v>
       </c>
     </row>
     <row r="170">
@@ -4450,7 +4450,7 @@
         <v>2.629999999999995</v>
       </c>
       <c r="E177" t="n">
-        <v>0.003483397570892999</v>
+        <v>0.003483397570893095</v>
       </c>
     </row>
     <row r="178">
@@ -4488,7 +4488,7 @@
         <v>344.9700000000012</v>
       </c>
       <c r="E179" t="n">
-        <v>0.01118110624141488</v>
+        <v>0.01118110624141496</v>
       </c>
     </row>
     <row r="180">
@@ -4545,7 +4545,7 @@
         <v>-38.15999999999985</v>
       </c>
       <c r="E182" t="n">
-        <v>-0.01722869100776092</v>
+        <v>-0.01722869100776097</v>
       </c>
     </row>
     <row r="183">
@@ -4583,7 +4583,7 @@
         <v>459</v>
       </c>
       <c r="E184" t="n">
-        <v>0.3348214285714286</v>
+        <v>0.3348214285714285</v>
       </c>
     </row>
     <row r="185">
@@ -4602,7 +4602,7 @@
         <v>-454.9299999999999</v>
       </c>
       <c r="E185" t="n">
-        <v>-0.5441420967645476</v>
+        <v>-0.5441420967645475</v>
       </c>
     </row>
     <row r="186">
@@ -4729,7 +4729,7 @@
         <v>-292.4200000000001</v>
       </c>
       <c r="E192" t="n">
-        <v>-0.03483807479189727</v>
+        <v>-0.03483807479189725</v>
       </c>
     </row>
     <row r="193">
@@ -4782,7 +4782,7 @@
         <v>1347.5</v>
       </c>
       <c r="E195" t="n">
-        <v>-13.68020304568528</v>
+        <v>13.68020304568528</v>
       </c>
     </row>
     <row r="196">
@@ -4820,7 +4820,7 @@
         <v>19909.42</v>
       </c>
       <c r="E197" t="n">
-        <v>4.353917546514578</v>
+        <v>4.353917546514577</v>
       </c>
     </row>
     <row r="198">
@@ -4890,7 +4890,7 @@
         <v>-4583.110000000001</v>
       </c>
       <c r="E201" t="n">
-        <v>-0.04954726369019768</v>
+        <v>-0.04954726369019769</v>
       </c>
     </row>
     <row r="202">
@@ -4909,7 +4909,7 @@
         <v>-2147.700000000001</v>
       </c>
       <c r="E202" t="n">
-        <v>-0.244604677066475</v>
+        <v>-0.2446046770664751</v>
       </c>
     </row>
     <row r="203">
@@ -4928,7 +4928,7 @@
         <v>-2191</v>
       </c>
       <c r="E203" t="n">
-        <v>-0.5757395796654352</v>
+        <v>-0.5757395796654351</v>
       </c>
     </row>
     <row r="204">
@@ -4998,7 +4998,7 @@
         <v>-4448.039999999999</v>
       </c>
       <c r="E207" t="n">
-        <v>-0.2189433518705016</v>
+        <v>-0.2189433518705017</v>
       </c>
     </row>
     <row r="208">
@@ -5034,7 +5034,7 @@
         <v>10.06999999999999</v>
       </c>
       <c r="E209" t="n">
-        <v>0.02135646420088233</v>
+        <v>0.02135646420088224</v>
       </c>
     </row>
     <row r="210">
@@ -5072,7 +5072,7 @@
         <v>237.24</v>
       </c>
       <c r="E211" t="n">
-        <v>0.5668952663146072</v>
+        <v>0.5668952663146073</v>
       </c>
     </row>
     <row r="212">
@@ -5108,7 +5108,7 @@
         <v>-9</v>
       </c>
       <c r="E213" t="n">
-        <v>-0.0007194819729794411</v>
+        <v>-0.0007194819729794548</v>
       </c>
     </row>
     <row r="214">
@@ -5273,7 +5273,7 @@
         <v>9626.889999999999</v>
       </c>
       <c r="E222" t="n">
-        <v>0.09073586334741957</v>
+        <v>0.09073586334741968</v>
       </c>
     </row>
     <row r="223">
@@ -5292,7 +5292,7 @@
         <v>177.4</v>
       </c>
       <c r="E223" t="n">
-        <v>0.4297272418971949</v>
+        <v>0.429727241897195</v>
       </c>
     </row>
     <row r="224">
@@ -5404,7 +5404,7 @@
         <v>-2464</v>
       </c>
       <c r="E229" t="n">
-        <v>-0.4338738561067217</v>
+        <v>-0.4338738561067216</v>
       </c>
     </row>
     <row r="230">
@@ -5423,7 +5423,7 @@
         <v>109.68</v>
       </c>
       <c r="E230" t="n">
-        <v>0.2228951165484585</v>
+        <v>0.2228951165484586</v>
       </c>
     </row>
     <row r="231">
@@ -5442,7 +5442,7 @@
         <v>864.5499999999993</v>
       </c>
       <c r="E231" t="n">
-        <v>-0.05518441827689036</v>
+        <v>0.05518441827689035</v>
       </c>
     </row>
     <row r="232">
@@ -5499,7 +5499,7 @@
         <v>-74.81999999999971</v>
       </c>
       <c r="E234" t="n">
-        <v>-0.03561212201982877</v>
+        <v>-0.0356121220198288</v>
       </c>
     </row>
     <row r="235">
@@ -5571,7 +5571,7 @@
         <v>1612.5</v>
       </c>
       <c r="E238" t="n">
-        <v>0.03527481542247735</v>
+        <v>0.03527481542247744</v>
       </c>
     </row>
     <row r="239">
@@ -5626,7 +5626,7 @@
         <v>199</v>
       </c>
       <c r="E241" t="n">
-        <v>0.05145748809883965</v>
+        <v>0.05145748809883975</v>
       </c>
     </row>
     <row r="242">
@@ -5719,7 +5719,7 @@
         <v>-408.9</v>
       </c>
       <c r="E246" t="n">
-        <v>-0.8194388777555111</v>
+        <v>-0.8194388777555109</v>
       </c>
     </row>
     <row r="247">
@@ -5869,7 +5869,7 @@
         <v>-144.5</v>
       </c>
       <c r="E254" t="n">
-        <v>-0.07896692679301376</v>
+        <v>-0.07896692679301374</v>
       </c>
     </row>
     <row r="255">
@@ -5926,7 +5926,7 @@
         <v>3.400000000000091</v>
       </c>
       <c r="E257" t="n">
-        <v>0.001624563398586742</v>
+        <v>0.001624563398586673</v>
       </c>
     </row>
     <row r="258">
@@ -6178,7 +6178,7 @@
         <v>12954.55</v>
       </c>
       <c r="E271" t="n">
-        <v>0.1473503596872721</v>
+        <v>0.147350359687272</v>
       </c>
     </row>
     <row r="272">
@@ -6197,7 +6197,7 @@
         <v>2050.59</v>
       </c>
       <c r="E272" t="n">
-        <v>0.3091688164050546</v>
+        <v>0.3091688164050544</v>
       </c>
     </row>
     <row r="273">
@@ -6286,7 +6286,7 @@
         <v>1129.359999999999</v>
       </c>
       <c r="E277" t="n">
-        <v>0.07117261893508275</v>
+        <v>0.0711726189350827</v>
       </c>
     </row>
     <row r="278">
@@ -6322,7 +6322,7 @@
         <v>-4.060000000000002</v>
       </c>
       <c r="E279" t="n">
-        <v>-0.008430407608131407</v>
+        <v>-0.008430407608131404</v>
       </c>
     </row>
     <row r="280">
@@ -6453,7 +6453,7 @@
         <v>374.64</v>
       </c>
       <c r="E286" t="n">
-        <v>-37464</v>
+        <v>37464</v>
       </c>
     </row>
     <row r="287">
@@ -6527,7 +6527,7 @@
         <v>-0.03999999999996362</v>
       </c>
       <c r="E290" t="n">
-        <v>-2.648831203233559e-05</v>
+        <v>-2.648831203229165e-05</v>
       </c>
     </row>
     <row r="291">
@@ -6601,7 +6601,7 @@
         <v>3494.91</v>
       </c>
       <c r="E294" t="n">
-        <v>-1.086418333120914</v>
+        <v>1.086418333120914</v>
       </c>
     </row>
     <row r="295">
@@ -6711,7 +6711,7 @@
         <v>95.03999999999996</v>
       </c>
       <c r="E300" t="n">
-        <v>0.1579393435812213</v>
+        <v>0.1579393435812214</v>
       </c>
     </row>
     <row r="301">
@@ -6730,7 +6730,7 @@
         <v>-431.7199999999993</v>
       </c>
       <c r="E301" t="n">
-        <v>0.02916630917017349</v>
+        <v>-0.02916630917017347</v>
       </c>
     </row>
     <row r="302">
@@ -6787,7 +6787,7 @@
         <v>108.5899999999997</v>
       </c>
       <c r="E304" t="n">
-        <v>0.05359425511437932</v>
+        <v>0.05359425511437933</v>
       </c>
     </row>
     <row r="305">
@@ -6859,7 +6859,7 @@
         <v>-30325</v>
       </c>
       <c r="E308" t="n">
-        <v>-0.6407818277865822</v>
+        <v>-0.6407818277865821</v>
       </c>
     </row>
     <row r="309">
@@ -6878,7 +6878,7 @@
         <v>611.4499999999998</v>
       </c>
       <c r="E309" t="n">
-        <v>0.09263088685988174</v>
+        <v>0.09263088685988183</v>
       </c>
     </row>
     <row r="310">
@@ -6914,7 +6914,7 @@
         <v>226.2999999999997</v>
       </c>
       <c r="E311" t="n">
-        <v>0.05565296942898512</v>
+        <v>0.05565296942898522</v>
       </c>
     </row>
     <row r="312">
@@ -7117,7 +7117,7 @@
         <v>-714.3500000000004</v>
       </c>
       <c r="E322" t="n">
-        <v>-0.2470705016463297</v>
+        <v>-0.2470705016463298</v>
       </c>
     </row>
     <row r="323">
@@ -7155,7 +7155,7 @@
         <v>-161.5</v>
       </c>
       <c r="E324" t="n">
-        <v>-0.09582408714948554</v>
+        <v>-0.09582408714948557</v>
       </c>
     </row>
     <row r="325">
@@ -7265,7 +7265,7 @@
         <v>-916.0499999999997</v>
       </c>
       <c r="E330" t="n">
-        <v>-0.2126935847129026</v>
+        <v>-0.2126935847129025</v>
       </c>
     </row>
     <row r="331">
@@ -7301,7 +7301,7 @@
         <v>-351.7100000000009</v>
       </c>
       <c r="E332" t="n">
-        <v>-0.03540488466811764</v>
+        <v>-0.03540488466811768</v>
       </c>
     </row>
     <row r="333">
@@ -7462,7 +7462,7 @@
         <v>2045.449999999997</v>
       </c>
       <c r="E341" t="n">
-        <v>0.02027783946260175</v>
+        <v>0.02027783946260179</v>
       </c>
     </row>
     <row r="342">
@@ -7481,7 +7481,7 @@
         <v>13.81999999999971</v>
       </c>
       <c r="E342" t="n">
-        <v>0.001591582807220382</v>
+        <v>0.001591582807220363</v>
       </c>
     </row>
     <row r="343">
@@ -7570,7 +7570,7 @@
         <v>-426.7599999999984</v>
       </c>
       <c r="E347" t="n">
-        <v>-0.02510757616227544</v>
+        <v>-0.02510757616227547</v>
       </c>
     </row>
     <row r="348">
@@ -7625,7 +7625,7 @@
         <v>358.02</v>
       </c>
       <c r="E350" t="n">
-        <v>0.1194750067576362</v>
+        <v>0.1194750067576361</v>
       </c>
     </row>
     <row r="351">
@@ -7807,7 +7807,7 @@
         <v>0.03999999999996362</v>
       </c>
       <c r="E360" t="n">
-        <v>2.648901368162981e-05</v>
+        <v>2.648901368155148e-05</v>
       </c>
     </row>
     <row r="361">
@@ -7843,7 +7843,7 @@
         <v>-7233.330000000002</v>
       </c>
       <c r="E362" t="n">
-        <v>-0.05910084531678428</v>
+        <v>-0.05910084531678424</v>
       </c>
     </row>
     <row r="363">
@@ -7970,7 +7970,7 @@
         <v>40.05999999999995</v>
       </c>
       <c r="E369" t="n">
-        <v>0.01246007085382272</v>
+        <v>0.01246007085382276</v>
       </c>
     </row>
     <row r="370">
@@ -7989,7 +7989,7 @@
         <v>-12.58999999999992</v>
       </c>
       <c r="E370" t="n">
-        <v>-0.01806857159258879</v>
+        <v>-0.01806857159258875</v>
       </c>
     </row>
     <row r="371">
@@ -8008,7 +8008,7 @@
         <v>1838.25</v>
       </c>
       <c r="E371" t="n">
-        <v>-0.1206697243550988</v>
+        <v>0.1206697243550989</v>
       </c>
     </row>
     <row r="372">
@@ -8137,7 +8137,7 @@
         <v>3787.5</v>
       </c>
       <c r="E378" t="n">
-        <v>0.2227941176470589</v>
+        <v>0.2227941176470588</v>
       </c>
     </row>
     <row r="379">
@@ -8156,7 +8156,7 @@
         <v>-1170.29</v>
       </c>
       <c r="E379" t="n">
-        <v>-0.1622612785238714</v>
+        <v>-0.1622612785238715</v>
       </c>
     </row>
     <row r="380">
@@ -8192,7 +8192,7 @@
         <v>-298.9999999999995</v>
       </c>
       <c r="E381" t="n">
-        <v>-0.06965524149868252</v>
+        <v>-0.0696552414986825</v>
       </c>
     </row>
     <row r="382">
@@ -8228,7 +8228,7 @@
         <v>2374</v>
       </c>
       <c r="E383" t="n">
-        <v>0.3646137306097375</v>
+        <v>0.3646137306097373</v>
       </c>
     </row>
     <row r="384">
@@ -8397,7 +8397,7 @@
         <v>33.43000000000029</v>
       </c>
       <c r="E392" t="n">
-        <v>0.01535648826558522</v>
+        <v>0.01535648826558516</v>
       </c>
     </row>
     <row r="393">
@@ -8454,7 +8454,7 @@
         <v>-64.80000000000001</v>
       </c>
       <c r="E395" t="n">
-        <v>-0.3710915129996565</v>
+        <v>-0.3710915129996564</v>
       </c>
     </row>
     <row r="396">
@@ -8490,7 +8490,7 @@
         <v>-192.48</v>
       </c>
       <c r="E397" t="n">
-        <v>-0.0778710079375996</v>
+        <v>-0.07787100793759963</v>
       </c>
     </row>
     <row r="398">
@@ -8579,7 +8579,7 @@
         <v>-790.7700000000004</v>
       </c>
       <c r="E402" t="n">
-        <v>-0.08252463153149114</v>
+        <v>-0.08252463153149116</v>
       </c>
     </row>
     <row r="403">
@@ -8670,7 +8670,7 @@
         <v>2899.31</v>
       </c>
       <c r="E407" t="n">
-        <v>0.5289205992454702</v>
+        <v>0.5289205992454703</v>
       </c>
     </row>
     <row r="408">
@@ -8759,7 +8759,7 @@
         <v>510.9500000000007</v>
       </c>
       <c r="E412" t="n">
-        <v>0.05875014372772225</v>
+        <v>0.05875014372772229</v>
       </c>
     </row>
     <row r="413">
@@ -8848,7 +8848,7 @@
         <v>1208.560000000001</v>
       </c>
       <c r="E417" t="n">
-        <v>0.07293443167074032</v>
+        <v>0.07293443167074025</v>
       </c>
     </row>
     <row r="418">
@@ -8903,7 +8903,7 @@
         <v>2403.09</v>
       </c>
       <c r="E420" t="n">
-        <v>0.7163502383273268</v>
+        <v>0.7163502383273267</v>
       </c>
     </row>
     <row r="421">
@@ -8922,7 +8922,7 @@
         <v>-4.319999999999993</v>
       </c>
       <c r="E421" t="n">
-        <v>-0.009578926362003526</v>
+        <v>-0.009578926362003576</v>
       </c>
     </row>
     <row r="422">
@@ -8977,7 +8977,7 @@
         <v>1500</v>
       </c>
       <c r="E424" t="n">
-        <v>0.2758620689655173</v>
+        <v>0.2758620689655172</v>
       </c>
     </row>
     <row r="425">
@@ -9087,7 +9087,7 @@
         <v>0.009999999999990905</v>
       </c>
       <c r="E430" t="n">
-        <v>6.622078008167165e-06</v>
+        <v>6.622078008072913e-06</v>
       </c>
     </row>
     <row r="431">
@@ -9123,7 +9123,7 @@
         <v>5891.670000000013</v>
       </c>
       <c r="E432" t="n">
-        <v>0.05116238114305371</v>
+        <v>0.05116238114305361</v>
       </c>
     </row>
     <row r="433">
@@ -9142,7 +9142,7 @@
         <v>33.79000000000002</v>
       </c>
       <c r="E433" t="n">
-        <v>0.07817235396182776</v>
+        <v>0.07817235396182769</v>
       </c>
     </row>
     <row r="434">
@@ -9161,7 +9161,7 @@
         <v>-21454.17</v>
       </c>
       <c r="E434" t="n">
-        <v>-0.9884436765722184</v>
+        <v>-0.9884436765722183</v>
       </c>
     </row>
     <row r="435">
@@ -9216,7 +9216,7 @@
         <v>352.9500000000007</v>
       </c>
       <c r="E437" t="n">
-        <v>0.01540714678586719</v>
+        <v>0.0154071467858671</v>
       </c>
     </row>
     <row r="438">
@@ -9252,7 +9252,7 @@
         <v>311.7399999999998</v>
       </c>
       <c r="E439" t="n">
-        <v>0.09576883258118718</v>
+        <v>0.09576883258118717</v>
       </c>
     </row>
     <row r="440">
@@ -9271,7 +9271,7 @@
         <v>74.65999999999997</v>
       </c>
       <c r="E440" t="n">
-        <v>0.109120140309851</v>
+        <v>0.1091201403098509</v>
       </c>
     </row>
     <row r="441">
@@ -9290,7 +9290,7 @@
         <v>1016.66</v>
       </c>
       <c r="E441" t="n">
-        <v>-0.07589574990967096</v>
+        <v>0.07589574990967102</v>
       </c>
     </row>
     <row r="442">
@@ -9438,7 +9438,7 @@
         <v>935.8099999999995</v>
       </c>
       <c r="E449" t="n">
-        <v>0.1548818372450591</v>
+        <v>0.1548818372450592</v>
       </c>
     </row>
     <row r="450">
@@ -9493,7 +9493,7 @@
         <v>-18.77000000000001</v>
       </c>
       <c r="E452" t="n">
-        <v>-0.08283684187298646</v>
+        <v>-0.0828368418729865</v>
       </c>
     </row>
     <row r="453">
@@ -9567,7 +9567,7 @@
         <v>117.5699999999999</v>
       </c>
       <c r="E456" t="n">
-        <v>0.2283533387717047</v>
+        <v>0.2283533387717048</v>
       </c>
     </row>
     <row r="457">
@@ -9624,7 +9624,7 @@
         <v>-531.25</v>
       </c>
       <c r="E459" t="n">
-        <v>-0.01702838427317732</v>
+        <v>-0.01702838427317727</v>
       </c>
     </row>
     <row r="460">
@@ -9679,7 +9679,7 @@
         <v>60.42000000000007</v>
       </c>
       <c r="E462" t="n">
-        <v>0.02733491376970276</v>
+        <v>0.0273349137697027</v>
       </c>
     </row>
     <row r="463">
@@ -9717,7 +9717,7 @@
         <v>306</v>
       </c>
       <c r="E464" t="n">
-        <v>0.2232142857142856</v>
+        <v>0.2232142857142857</v>
       </c>
     </row>
     <row r="465">
@@ -9827,7 +9827,7 @@
         <v>574.6199999999999</v>
       </c>
       <c r="E470" t="n">
-        <v>0.1694619343232522</v>
+        <v>0.1694619343232523</v>
       </c>
     </row>
     <row r="471">
@@ -9863,7 +9863,7 @@
         <v>419.7100000000009</v>
       </c>
       <c r="E472" t="n">
-        <v>0.04774064831097458</v>
+        <v>0.04774064831097462</v>
       </c>
     </row>
     <row r="473">
@@ -9954,7 +9954,7 @@
         <v>-903.0300000000007</v>
       </c>
       <c r="E477" t="n">
-        <v>-0.1077489568505419</v>
+        <v>-0.1077489568505418</v>
       </c>
     </row>
     <row r="478">
@@ -10024,7 +10024,7 @@
         <v>-9583.329999999987</v>
       </c>
       <c r="E481" t="n">
-        <v>-0.09311739159795807</v>
+        <v>-0.09311739159795804</v>
       </c>
     </row>
     <row r="482">
@@ -10132,7 +10132,7 @@
         <v>44.70999999999913</v>
       </c>
       <c r="E487" t="n">
-        <v>0.002514756123214612</v>
+        <v>0.002514756123214564</v>
       </c>
     </row>
     <row r="488">
@@ -10168,7 +10168,7 @@
         <v>-0.2199999999999704</v>
       </c>
       <c r="E489" t="n">
-        <v>-0.0004607040395366857</v>
+        <v>-0.0004607040395367212</v>
       </c>
     </row>
     <row r="490">
@@ -10206,7 +10206,7 @@
         <v>-5.910000000000025</v>
       </c>
       <c r="E491" t="n">
-        <v>-0.01323124454295121</v>
+        <v>-0.01323124454295123</v>
       </c>
     </row>
     <row r="492">
@@ -10367,7 +10367,7 @@
         <v>-0.02999999999997272</v>
       </c>
       <c r="E500" t="n">
-        <v>-1.986610246929033e-05</v>
+        <v>-1.986610246933847e-05</v>
       </c>
     </row>
     <row r="501">
@@ -10422,7 +10422,7 @@
         <v>24.13999999999999</v>
       </c>
       <c r="E503" t="n">
-        <v>0.0517981289159728</v>
+        <v>0.05179812891597285</v>
       </c>
     </row>
     <row r="504">
@@ -10496,7 +10496,7 @@
         <v>-15090.52</v>
       </c>
       <c r="E507" t="n">
-        <v>-0.6487435058025937</v>
+        <v>-0.6487435058025935</v>
       </c>
     </row>
     <row r="508">
@@ -10551,7 +10551,7 @@
         <v>33.88</v>
       </c>
       <c r="E510" t="n">
-        <v>0.04464591624278524</v>
+        <v>0.04464591624278522</v>
       </c>
     </row>
     <row r="511">
@@ -10570,7 +10570,7 @@
         <v>1213.789999999999</v>
       </c>
       <c r="E511" t="n">
-        <v>-0.09805377249204683</v>
+        <v>0.09805377249204683</v>
       </c>
     </row>
     <row r="512">
@@ -10646,7 +10646,7 @@
         <v>-36.94000000000005</v>
       </c>
       <c r="E515" t="n">
-        <v>-0.0417887484869397</v>
+        <v>-0.04178874848693966</v>
       </c>
     </row>
     <row r="516">
@@ -10773,7 +10773,7 @@
         <v>-34.10999999999999</v>
       </c>
       <c r="E522" t="n">
-        <v>-0.1641324222885189</v>
+        <v>-0.1641324222885188</v>
       </c>
     </row>
     <row r="523">
@@ -10826,7 +10826,7 @@
         <v>-288.9299999999998</v>
       </c>
       <c r="E525" t="n">
-        <v>-0.1364209393133862</v>
+        <v>-0.1364209393133861</v>
       </c>
     </row>
     <row r="526">
@@ -10845,7 +10845,7 @@
         <v>347.3900000000001</v>
       </c>
       <c r="E526" t="n">
-        <v>0.5492939930110845</v>
+        <v>0.5492939930110844</v>
       </c>
     </row>
     <row r="527">
@@ -11143,7 +11143,7 @@
         <v>-490.3199999999997</v>
       </c>
       <c r="E542" t="n">
-        <v>-0.05323102276909442</v>
+        <v>-0.05323102276909445</v>
       </c>
     </row>
     <row r="543">
@@ -11196,7 +11196,7 @@
         <v>150</v>
       </c>
       <c r="E545" t="n">
-        <v>0.03158559696778274</v>
+        <v>0.03158559696778269</v>
       </c>
     </row>
     <row r="546">
@@ -11234,7 +11234,7 @@
         <v>1996.01</v>
       </c>
       <c r="E547" t="n">
-        <v>0.2669233361505461</v>
+        <v>0.2669233361505462</v>
       </c>
     </row>
     <row r="548">
@@ -11304,7 +11304,7 @@
         <v>-3958.330000000002</v>
       </c>
       <c r="E551" t="n">
-        <v>-0.04241068463009778</v>
+        <v>-0.04241068463009782</v>
       </c>
     </row>
     <row r="552">
@@ -11342,7 +11342,7 @@
         <v>-78.72000000000025</v>
       </c>
       <c r="E553" t="n">
-        <v>-0.02835009777758579</v>
+        <v>-0.0283500977775858</v>
       </c>
     </row>
     <row r="554">
@@ -11469,7 +11469,7 @@
         <v>2271.51</v>
       </c>
       <c r="E560" t="n">
-        <v>0.4436283030291195</v>
+        <v>0.4436283030291194</v>
       </c>
     </row>
     <row r="561">
@@ -11488,7 +11488,7 @@
         <v>-34.31</v>
       </c>
       <c r="E561" t="n">
-        <v>-0.07784281695253659</v>
+        <v>-0.07784281695253653</v>
       </c>
     </row>
     <row r="562">
@@ -11706,7 +11706,7 @@
         <v>-57.93000000000001</v>
       </c>
       <c r="E573" t="n">
-        <v>-0.118181076339304</v>
+        <v>-0.1181810763393039</v>
       </c>
     </row>
     <row r="574">
@@ -11835,7 +11835,7 @@
         <v>-14.76999999999998</v>
       </c>
       <c r="E580" t="n">
-        <v>-0.01863158160304768</v>
+        <v>-0.01863158160304763</v>
       </c>
     </row>
     <row r="581">
@@ -11854,7 +11854,7 @@
         <v>1293.450000000001</v>
       </c>
       <c r="E581" t="n">
-        <v>-0.1158483228437363</v>
+        <v>0.1158483228437363</v>
       </c>
     </row>
     <row r="582">
@@ -11930,7 +11930,7 @@
         <v>36.94000000000005</v>
       </c>
       <c r="E585" t="n">
-        <v>0.04361120621465608</v>
+        <v>0.04361120621465598</v>
       </c>
     </row>
     <row r="586">
@@ -12002,7 +12002,7 @@
         <v>-444.3399999999992</v>
       </c>
       <c r="E589" t="n">
-        <v>-0.0766485369434079</v>
+        <v>-0.07664853694340788</v>
       </c>
     </row>
     <row r="590">
@@ -12040,7 +12040,7 @@
         <v>106.9400000000001</v>
       </c>
       <c r="E591" t="n">
-        <v>0.02677804570847631</v>
+        <v>0.02677804570847639</v>
       </c>
     </row>
     <row r="592">
@@ -12152,7 +12152,7 @@
         <v>11.91999999999996</v>
       </c>
       <c r="E597" t="n">
-        <v>0.01793317185454857</v>
+        <v>0.01793317185454867</v>
       </c>
     </row>
     <row r="598">
@@ -12209,7 +12209,7 @@
         <v>67.50999999999999</v>
       </c>
       <c r="E600" t="n">
-        <v>0.1176050449446031</v>
+        <v>0.1176050449446032</v>
       </c>
     </row>
     <row r="601">
@@ -12245,7 +12245,7 @@
         <v>-8.319999999999709</v>
       </c>
       <c r="E602" t="n">
-        <v>-0.003794581775061423</v>
+        <v>-0.003794581775061438</v>
       </c>
     </row>
     <row r="603">
@@ -12302,7 +12302,7 @@
         <v>30</v>
       </c>
       <c r="E605" t="n">
-        <v>0.0372754156208841</v>
+        <v>0.03727541562088417</v>
       </c>
     </row>
     <row r="606">
@@ -12611,7 +12611,7 @@
         <v>176.4499999999998</v>
       </c>
       <c r="E622" t="n">
-        <v>0.02637159967777181</v>
+        <v>0.02637159967777176</v>
       </c>
     </row>
     <row r="623">
@@ -12630,7 +12630,7 @@
         <v>-263.4599999999996</v>
       </c>
       <c r="E623" t="n">
-        <v>-0.09765047312999664</v>
+        <v>-0.09765047312999663</v>
       </c>
     </row>
     <row r="624">
@@ -12700,7 +12700,7 @@
         <v>-302.6699999999983</v>
       </c>
       <c r="E627" t="n">
-        <v>-0.01448428536152557</v>
+        <v>-0.01448428536152561</v>
       </c>
     </row>
     <row r="628">
@@ -12774,7 +12774,7 @@
         <v>17.44</v>
       </c>
       <c r="E631" t="n">
-        <v>0.04290810677820156</v>
+        <v>0.0429081067782015</v>
       </c>
     </row>
     <row r="632">
@@ -12975,7 +12975,7 @@
         <v>353.0299999999988</v>
       </c>
       <c r="E642" t="n">
-        <v>0.002916447332115268</v>
+        <v>0.002916447332115294</v>
       </c>
     </row>
     <row r="643">
@@ -13013,7 +13013,7 @@
         <v>995.3199999999997</v>
       </c>
       <c r="E644" t="n">
-        <v>0.0382037350856621</v>
+        <v>0.03820373508566207</v>
       </c>
     </row>
     <row r="645">
@@ -13049,7 +13049,7 @@
         <v>-27.78999999999999</v>
       </c>
       <c r="E646" t="n">
-        <v>-0.1098766408350467</v>
+        <v>-0.1098766408350466</v>
       </c>
     </row>
     <row r="647">
@@ -13123,7 +13123,7 @@
         <v>37.02999999999997</v>
       </c>
       <c r="E650" t="n">
-        <v>0.04759823643585226</v>
+        <v>0.04759823643585225</v>
       </c>
     </row>
     <row r="651">
@@ -13142,7 +13142,7 @@
         <v>1429.76</v>
       </c>
       <c r="E651" t="n">
-        <v>-0.1448359837027102</v>
+        <v>0.1448359837027102</v>
       </c>
     </row>
     <row r="652">
@@ -13161,7 +13161,7 @@
         <v>-675</v>
       </c>
       <c r="E652" t="n">
-        <v>-0.3333333333333334</v>
+        <v>-0.3333333333333333</v>
       </c>
     </row>
     <row r="653">
@@ -13180,7 +13180,7 @@
         <v>37.02000000000044</v>
       </c>
       <c r="E653" t="n">
-        <v>0.001388250347062581</v>
+        <v>0.001388250347062603</v>
       </c>
     </row>
     <row r="654">
@@ -13199,7 +13199,7 @@
         <v>296.3100000000004</v>
       </c>
       <c r="E654" t="n">
-        <v>0.1388037887517919</v>
+        <v>0.138803788751792</v>
       </c>
     </row>
     <row r="655">
@@ -13271,7 +13271,7 @@
         <v>2275</v>
       </c>
       <c r="E658" t="n">
-        <v>0.2492557934167985</v>
+        <v>0.2492557934167984</v>
       </c>
     </row>
     <row r="659">
@@ -13290,7 +13290,7 @@
         <v>491.7399999999998</v>
       </c>
       <c r="E659" t="n">
-        <v>0.0918664541910077</v>
+        <v>0.0918664541910076</v>
       </c>
     </row>
     <row r="660">
@@ -13326,7 +13326,7 @@
         <v>64.28999999999996</v>
       </c>
       <c r="E661" t="n">
-        <v>0.01567853754776838</v>
+        <v>0.01567853754776844</v>
       </c>
     </row>
     <row r="662">
@@ -13402,7 +13402,7 @@
         <v>86.56</v>
       </c>
       <c r="E665" t="n">
-        <v>1.095696202531645</v>
+        <v>1.095696202531646</v>
       </c>
     </row>
     <row r="666">
@@ -13440,7 +13440,7 @@
         <v>-55.40999999999997</v>
       </c>
       <c r="E667" t="n">
-        <v>-0.08189355758856653</v>
+        <v>-0.08189355758856648</v>
       </c>
     </row>
     <row r="668">
@@ -13478,7 +13478,7 @@
         <v>10.7400000000016</v>
       </c>
       <c r="E669" t="n">
-        <v>0.0003502174674385738</v>
+        <v>0.0003502174674386321</v>
       </c>
     </row>
     <row r="670">
@@ -13497,7 +13497,7 @@
         <v>-33.99000000000001</v>
       </c>
       <c r="E670" t="n">
-        <v>-0.05298106149169979</v>
+        <v>-0.05298106149169981</v>
       </c>
     </row>
     <row r="671">
@@ -13533,7 +13533,7 @@
         <v>2.9699999999998</v>
       </c>
       <c r="E672" t="n">
-        <v>0.001359715787353277</v>
+        <v>0.001359715787353178</v>
       </c>
     </row>
     <row r="673">
@@ -13719,7 +13719,7 @@
         <v>-790.79</v>
       </c>
       <c r="E682" t="n">
-        <v>-0.1026021947909396</v>
+        <v>-0.1026021947909395</v>
       </c>
     </row>
     <row r="683">
@@ -13772,7 +13772,7 @@
         <v>-150</v>
       </c>
       <c r="E685" t="n">
-        <v>-0.03061849357011637</v>
+        <v>-0.03061849357011635</v>
       </c>
     </row>
     <row r="686">
@@ -13810,7 +13810,7 @@
         <v>-1966.299999999999</v>
       </c>
       <c r="E687" t="n">
-        <v>-0.09768041915694681</v>
+        <v>-0.09768041915694686</v>
       </c>
     </row>
     <row r="688">
@@ -13880,7 +13880,7 @@
         <v>80.27999999999884</v>
       </c>
       <c r="E691" t="n">
-        <v>0.0009398634879893564</v>
+        <v>0.0009398634879893318</v>
       </c>
     </row>
     <row r="692">
@@ -13918,7 +13918,7 @@
         <v>61.61999999999989</v>
       </c>
       <c r="E693" t="n">
-        <v>0.02531084028539388</v>
+        <v>0.02531084028539385</v>
       </c>
     </row>
     <row r="694">
@@ -13988,7 +13988,7 @@
         <v>3038.649999999998</v>
       </c>
       <c r="E697" t="n">
-        <v>0.1475519052606686</v>
+        <v>0.1475519052606685</v>
       </c>
     </row>
     <row r="698">
@@ -14024,7 +14024,7 @@
         <v>1.139999999999986</v>
       </c>
       <c r="E699" t="n">
-        <v>0.002388384907083374</v>
+        <v>0.002388384907083418</v>
       </c>
     </row>
     <row r="700">
@@ -14043,7 +14043,7 @@
         <v>-194.1500000000001</v>
       </c>
       <c r="E700" t="n">
-        <v>-0.07432745426076437</v>
+        <v>-0.0743274542607644</v>
       </c>
     </row>
     <row r="701">
@@ -14062,7 +14062,7 @@
         <v>-31.57999999999998</v>
       </c>
       <c r="E701" t="n">
-        <v>-0.07450046002500643</v>
+        <v>-0.07450046002500645</v>
       </c>
     </row>
     <row r="702">
@@ -14153,7 +14153,7 @@
         <v>-16.38</v>
       </c>
       <c r="E706" t="n">
-        <v>-0.2763157894736843</v>
+        <v>-0.2763157894736842</v>
       </c>
     </row>
     <row r="707">
@@ -14225,7 +14225,7 @@
         <v>0.02999999999997272</v>
       </c>
       <c r="E710" t="n">
-        <v>1.986649713914268e-05</v>
+        <v>1.986649713920634e-05</v>
       </c>
     </row>
     <row r="711">
@@ -14261,7 +14261,7 @@
         <v>-353.0299999999988</v>
       </c>
       <c r="E712" t="n">
-        <v>-0.002907966401262452</v>
+        <v>-0.002907966401262451</v>
       </c>
     </row>
     <row r="713">
@@ -14299,7 +14299,7 @@
         <v>-26683.18</v>
       </c>
       <c r="E714" t="n">
-        <v>-0.9865022790736709</v>
+        <v>-0.9865022790736708</v>
       </c>
     </row>
     <row r="715">
@@ -14356,7 +14356,7 @@
         <v>872.869999999999</v>
       </c>
       <c r="E717" t="n">
-        <v>0.0383931925285308</v>
+        <v>0.03839319252853083</v>
       </c>
     </row>
     <row r="718">
@@ -14430,7 +14430,7 @@
         <v>412.3299999999999</v>
       </c>
       <c r="E721" t="n">
-        <v>-0.04884373274957299</v>
+        <v>0.04884373274957295</v>
       </c>
     </row>
     <row r="722">
@@ -14449,7 +14449,7 @@
         <v>-21.94000000000005</v>
       </c>
       <c r="E722" t="n">
-        <v>-0.01625185185185185</v>
+        <v>-0.01625185185185189</v>
       </c>
     </row>
     <row r="723">
@@ -14468,7 +14468,7 @@
         <v>-37.02000000000044</v>
       </c>
       <c r="E723" t="n">
-        <v>-0.001386325779817676</v>
+        <v>-0.001386325779817629</v>
       </c>
     </row>
     <row r="724">
@@ -14506,7 +14506,7 @@
         <v>-135.89</v>
       </c>
       <c r="E725" t="n">
-        <v>-0.1537269364344943</v>
+        <v>-0.1537269364344944</v>
       </c>
     </row>
     <row r="726">
@@ -14578,7 +14578,7 @@
         <v>492.1399999999994</v>
       </c>
       <c r="E729" t="n">
-        <v>0.08420551936774845</v>
+        <v>0.08420551936774844</v>
       </c>
     </row>
     <row r="730">
@@ -14616,7 +14616,7 @@
         <v>240.5699999999997</v>
       </c>
       <c r="E731" t="n">
-        <v>0.0577626776796003</v>
+        <v>0.05776267767960039</v>
       </c>
     </row>
     <row r="732">
@@ -14709,7 +14709,7 @@
         <v>-311.59</v>
       </c>
       <c r="E736" t="n">
-        <v>-0.8831665769110852</v>
+        <v>-0.8831665769110854</v>
       </c>
     </row>
     <row r="737">
@@ -14764,7 +14764,7 @@
         <v>-10.7400000000016</v>
       </c>
       <c r="E739" t="n">
-        <v>-0.0003500948581041108</v>
+        <v>-0.0003500948581040636</v>
       </c>
     </row>
     <row r="740">
@@ -14783,7 +14783,7 @@
         <v>-12.92999999999995</v>
       </c>
       <c r="E740" t="n">
-        <v>-0.02128184870630057</v>
+        <v>-0.02128184870630053</v>
       </c>
     </row>
     <row r="741">
@@ -14819,7 +14819,7 @@
         <v>14.34999999999991</v>
       </c>
       <c r="E742" t="n">
-        <v>0.006560749799977117</v>
+        <v>0.006560749799977099</v>
       </c>
     </row>
     <row r="743">
@@ -14857,7 +14857,7 @@
         <v>43.5</v>
       </c>
       <c r="E744" t="n">
-        <v>0.1506024096385543</v>
+        <v>0.1506024096385542</v>
       </c>
     </row>
     <row r="745">
@@ -14876,7 +14876,7 @@
         <v>-635.01</v>
       </c>
       <c r="E745" t="n">
-        <v>-0.8525684057893183</v>
+        <v>-0.8525684057893181</v>
       </c>
     </row>
     <row r="746">
@@ -14914,7 +14914,7 @@
         <v>182.3399999999997</v>
       </c>
       <c r="E747" t="n">
-        <v>0.07999824507524234</v>
+        <v>0.07999824507524225</v>
       </c>
     </row>
     <row r="748">
@@ -14969,7 +14969,7 @@
         <v>-353.0100000000002</v>
       </c>
       <c r="E750" t="n">
-        <v>-0.08811482059282372</v>
+        <v>-0.08811482059282377</v>
       </c>
     </row>
     <row r="751">
@@ -15005,7 +15005,7 @@
         <v>-385.9099999999999</v>
       </c>
       <c r="E752" t="n">
-        <v>-0.05579515799061674</v>
+        <v>-0.05579515799061668</v>
       </c>
     </row>
     <row r="753">
@@ -15058,7 +15058,7 @@
         <v>9.199999999999818</v>
       </c>
       <c r="E755" t="n">
-        <v>0.001937249947357333</v>
+        <v>0.0019372499473573</v>
       </c>
     </row>
     <row r="756">
@@ -15166,7 +15166,7 @@
         <v>-80.27999999999884</v>
       </c>
       <c r="E761" t="n">
-        <v>-0.0009389809740558697</v>
+        <v>-0.0009389809740558999</v>
       </c>
     </row>
     <row r="762">
@@ -15204,7 +15204,7 @@
         <v>-246.4000000000001</v>
       </c>
       <c r="E763" t="n">
-        <v>-0.09871201650541839</v>
+        <v>-0.09871201650541837</v>
       </c>
     </row>
     <row r="764">
@@ -15274,7 +15274,7 @@
         <v>-1246.739999999998</v>
       </c>
       <c r="E767" t="n">
-        <v>-0.05275549435902027</v>
+        <v>-0.05275549435902028</v>
       </c>
     </row>
     <row r="768">
@@ -15348,7 +15348,7 @@
         <v>24.69</v>
       </c>
       <c r="E771" t="n">
-        <v>0.06293492391221234</v>
+        <v>0.06293492391221228</v>
       </c>
     </row>
     <row r="772">
@@ -15439,7 +15439,7 @@
         <v>4.359999999999999</v>
       </c>
       <c r="E776" t="n">
-        <v>0.1016317016317017</v>
+        <v>0.1016317016317016</v>
       </c>
     </row>
     <row r="777">
@@ -15511,7 +15511,7 @@
         <v>-0.01999999999998181</v>
       </c>
       <c r="E780" t="n">
-        <v>-1.324406831293423e-05</v>
+        <v>-1.324406831289231e-05</v>
       </c>
     </row>
     <row r="781">
@@ -15676,7 +15676,7 @@
         <v>948.8100000000004</v>
       </c>
       <c r="E789" t="n">
-        <v>0.2944904667165342</v>
+        <v>0.2944904667165343</v>
       </c>
     </row>
     <row r="790">
@@ -15695,7 +15695,7 @@
         <v>22.32999999999993</v>
       </c>
       <c r="E790" t="n">
-        <v>0.02794953313139903</v>
+        <v>0.02794953313139901</v>
       </c>
     </row>
     <row r="791">
@@ -15714,7 +15714,7 @@
         <v>1184.849999999999</v>
       </c>
       <c r="E791" t="n">
-        <v>-0.1475622984772382</v>
+        <v>0.1475622984772382</v>
       </c>
     </row>
     <row r="792">
@@ -15771,7 +15771,7 @@
         <v>-0.3699999999998909</v>
       </c>
       <c r="E794" t="n">
-        <v>-0.0001733532611496447</v>
+        <v>-0.000173353261149609</v>
       </c>
     </row>
     <row r="795">
@@ -15790,7 +15790,7 @@
         <v>-62.04000000000008</v>
       </c>
       <c r="E795" t="n">
-        <v>-0.08293230670516527</v>
+        <v>-0.08293230670516533</v>
       </c>
     </row>
     <row r="796">
@@ -15862,7 +15862,7 @@
         <v>-752.6199999999999</v>
       </c>
       <c r="E799" t="n">
-        <v>-0.1187725375395516</v>
+        <v>-0.1187725375395517</v>
       </c>
     </row>
     <row r="800">
@@ -15881,7 +15881,7 @@
         <v>66.39999999999964</v>
       </c>
       <c r="E800" t="n">
-        <v>0.01327999999999996</v>
+        <v>0.01327999999999993</v>
       </c>
     </row>
     <row r="801">
@@ -16008,7 +16008,7 @@
         <v>-131.11</v>
       </c>
       <c r="E807" t="n">
-        <v>-0.2254453538757824</v>
+        <v>-0.2254453538757823</v>
       </c>
     </row>
     <row r="808">
@@ -16027,7 +16027,7 @@
         <v>-1452.69</v>
       </c>
       <c r="E808" t="n">
-        <v>-0.664527343839345</v>
+        <v>-0.6645273438393449</v>
       </c>
     </row>
     <row r="809">
@@ -16065,7 +16065,7 @@
         <v>-10.62</v>
       </c>
       <c r="E810" t="n">
-        <v>-0.01785984561828369</v>
+        <v>-0.01785984561828365</v>
       </c>
     </row>
     <row r="811">
@@ -16101,7 +16101,7 @@
         <v>17.32999999999993</v>
       </c>
       <c r="E812" t="n">
-        <v>0.007871547965116354</v>
+        <v>0.007871547965116247</v>
       </c>
     </row>
     <row r="813">
@@ -16196,7 +16196,7 @@
         <v>159.5300000000002</v>
       </c>
       <c r="E817" t="n">
-        <v>0.06480638923644411</v>
+        <v>0.06480638923644408</v>
       </c>
     </row>
     <row r="818">
@@ -16249,7 +16249,7 @@
         <v>353.0100000000002</v>
       </c>
       <c r="E820" t="n">
-        <v>0.09662929344910287</v>
+        <v>0.09662929344910277</v>
       </c>
     </row>
     <row r="821">
@@ -16484,7 +16484,7 @@
         <v>235.8400000000001</v>
       </c>
       <c r="E833" t="n">
-        <v>0.1048294254917215</v>
+        <v>0.1048294254917214</v>
       </c>
     </row>
     <row r="834">
@@ -16554,7 +16554,7 @@
         <v>2511.489999999998</v>
       </c>
       <c r="E837" t="n">
-        <v>0.1121918119083269</v>
+        <v>0.112191811908327</v>
       </c>
     </row>
     <row r="838">
@@ -16609,7 +16609,7 @@
         <v>4245.139999999999</v>
       </c>
       <c r="E840" t="n">
-        <v>3.100951073061696</v>
+        <v>3.100951073061695</v>
       </c>
     </row>
     <row r="841">
@@ -16628,7 +16628,7 @@
         <v>-21.06</v>
       </c>
       <c r="E841" t="n">
-        <v>-0.05050359712230212</v>
+        <v>-0.05050359712230217</v>
       </c>
     </row>
     <row r="842">
@@ -16791,7 +16791,7 @@
         <v>-1069.06</v>
       </c>
       <c r="E850" t="n">
-        <v>-0.7079445595957856</v>
+        <v>-0.7079445595957857</v>
       </c>
     </row>
     <row r="851">
@@ -16901,7 +16901,7 @@
         <v>10549.65</v>
       </c>
       <c r="E856" t="n">
-        <v>6.793296628996426</v>
+        <v>6.793296628996425</v>
       </c>
     </row>
     <row r="857">
@@ -16920,7 +16920,7 @@
         <v>-5698.940000000002</v>
       </c>
       <c r="E857" t="n">
-        <v>-0.2756753488304596</v>
+        <v>-0.2756753488304597</v>
       </c>
     </row>
     <row r="858">
@@ -16939,7 +16939,7 @@
         <v>1244429.84</v>
       </c>
       <c r="E858" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="859">
@@ -16977,7 +16977,7 @@
         <v>67.61000000000001</v>
       </c>
       <c r="E860" t="n">
-        <v>0.08232371814385031</v>
+        <v>0.08232371814385039</v>
       </c>
     </row>
     <row r="861">
@@ -16996,7 +16996,7 @@
         <v>1395.35</v>
       </c>
       <c r="E861" t="n">
-        <v>-0.2038602468500901</v>
+        <v>0.20386024685009</v>
       </c>
     </row>
     <row r="862">
@@ -17053,7 +17053,7 @@
         <v>947.8499999999999</v>
       </c>
       <c r="E864" t="n">
-        <v>0.4441658856607309</v>
+        <v>0.444165885660731</v>
       </c>
     </row>
     <row r="865">
@@ -17182,7 +17182,7 @@
         <v>8.340000000000146</v>
       </c>
       <c r="E871" t="n">
-        <v>0.002419467137021902</v>
+        <v>0.002419467137021951</v>
       </c>
     </row>
     <row r="872">
@@ -17252,7 +17252,7 @@
         <v>3251.03</v>
       </c>
       <c r="E875" t="n">
-        <v>0.8234333129017715</v>
+        <v>0.8234333129017716</v>
       </c>
     </row>
     <row r="876">
@@ -17402,7 +17402,7 @@
         <v>-8333.32</v>
       </c>
       <c r="E883" t="n">
-        <v>-0.4347820642720224</v>
+        <v>-0.4347820642720223</v>
       </c>
     </row>
     <row r="884">
@@ -17478,7 +17478,7 @@
         <v>165.8199999999997</v>
       </c>
       <c r="E887" t="n">
-        <v>0.06326182582587148</v>
+        <v>0.06326182582587155</v>
       </c>
     </row>
     <row r="888">
@@ -17531,7 +17531,7 @@
         <v>70.09999999999991</v>
       </c>
       <c r="E890" t="n">
-        <v>0.01749765990639629</v>
+        <v>0.01749765990639623</v>
       </c>
     </row>
     <row r="891">
@@ -17567,7 +17567,7 @@
         <v>8189.889999999999</v>
       </c>
       <c r="E892" t="n">
-        <v>1.481724250850781</v>
+        <v>1.481724250850782</v>
       </c>
     </row>
     <row r="893">
@@ -17622,7 +17622,7 @@
         <v>3400</v>
       </c>
       <c r="E895" t="n">
-        <v>0.7145559245092683</v>
+        <v>0.7145559245092682</v>
       </c>
     </row>
     <row r="896">
@@ -17768,7 +17768,7 @@
         <v>2122.71</v>
       </c>
       <c r="E903" t="n">
-        <v>0.8540064934281197</v>
+        <v>0.8540064934281196</v>
       </c>
     </row>
     <row r="904">
@@ -17838,7 +17838,7 @@
         <v>-605.1899999999987</v>
       </c>
       <c r="E907" t="n">
-        <v>-0.02430758194606053</v>
+        <v>-0.02430758194606049</v>
       </c>
     </row>
     <row r="908">
@@ -17876,7 +17876,7 @@
         <v>-0.7699999999999818</v>
       </c>
       <c r="E909" t="n">
-        <v>-0.001609363569860967</v>
+        <v>-0.001609363569860972</v>
       </c>
     </row>
     <row r="910">
@@ -17914,7 +17914,7 @@
         <v>-56.62</v>
       </c>
       <c r="E911" t="n">
-        <v>-0.1430014648684145</v>
+        <v>-0.1430014648684144</v>
       </c>
     </row>
     <row r="912">
@@ -17950,7 +17950,7 @@
         <v>1000</v>
       </c>
       <c r="E913" t="n">
-        <v>0.08000000000000007</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="914">
@@ -18079,7 +18079,7 @@
         <v>0.03000000000002956</v>
       </c>
       <c r="E920" t="n">
-        <v>6.802258349769552e-05</v>
+        <v>6.802258349778827e-05</v>
       </c>
     </row>
     <row r="921">
@@ -18282,7 +18282,7 @@
         <v>2015.01</v>
       </c>
       <c r="E931" t="n">
-        <v>-0.3697747779986016</v>
+        <v>0.3697747779986016</v>
       </c>
     </row>
     <row r="932">
@@ -18428,7 +18428,7 @@
         <v>75.38999999999942</v>
       </c>
       <c r="E939" t="n">
-        <v>0.01066333617160908</v>
+        <v>0.01066333617160905</v>
       </c>
     </row>
     <row r="940">
@@ -18464,7 +18464,7 @@
         <v>-163.2800000000002</v>
       </c>
       <c r="E941" t="n">
-        <v>-0.0472538476231269</v>
+        <v>-0.04725384762312689</v>
       </c>
     </row>
     <row r="942">
@@ -18555,7 +18555,7 @@
         <v>-2027.52</v>
       </c>
       <c r="E946" t="n">
-        <v>-0.6578884180332656</v>
+        <v>-0.6578884180332657</v>
       </c>
     </row>
     <row r="947">
@@ -18593,7 +18593,7 @@
         <v>-2364.48</v>
       </c>
       <c r="E948" t="n">
-        <v>-0.8762818208434168</v>
+        <v>-0.8762818208434169</v>
       </c>
     </row>
     <row r="949">
@@ -18612,7 +18612,7 @@
         <v>500</v>
       </c>
       <c r="E949" t="n">
-        <v>0.01630435137051123</v>
+        <v>0.01630435137051117</v>
       </c>
     </row>
     <row r="950">
@@ -18705,7 +18705,7 @@
         <v>-179.75</v>
       </c>
       <c r="E954" t="n">
-        <v>-0.09390689242632422</v>
+        <v>-0.09390689242632423</v>
       </c>
     </row>
     <row r="955">
@@ -18762,7 +18762,7 @@
         <v>-188.4299999999998</v>
       </c>
       <c r="E957" t="n">
-        <v>-0.06761057628480904</v>
+        <v>-0.067610576284809</v>
       </c>
     </row>
     <row r="958">
@@ -18815,7 +18815,7 @@
         <v>3.579999999999927</v>
       </c>
       <c r="E960" t="n">
-        <v>0.0008782366577944067</v>
+        <v>0.0008782366577943325</v>
       </c>
     </row>
     <row r="961">
@@ -18904,7 +18904,7 @@
         <v>1848.250000000001</v>
       </c>
       <c r="E965" t="n">
-        <v>0.2265512000196124</v>
+        <v>0.2265512000196123</v>
       </c>
     </row>
     <row r="966">
@@ -18923,7 +18923,7 @@
         <v>-5907.6</v>
       </c>
       <c r="E966" t="n">
-        <v>-0.4690123636155775</v>
+        <v>-0.4690123636155776</v>
       </c>
     </row>
     <row r="967">
@@ -19031,7 +19031,7 @@
         <v>-6848.74</v>
       </c>
       <c r="E972" t="n">
-        <v>-0.4641514293072366</v>
+        <v>-0.4641514293072367</v>
       </c>
     </row>
     <row r="973">
@@ -19120,7 +19120,7 @@
         <v>1051.959999999999</v>
       </c>
       <c r="E977" t="n">
-        <v>0.04330482735454244</v>
+        <v>0.04330482735454249</v>
       </c>
     </row>
     <row r="978">
@@ -19175,7 +19175,7 @@
         <v>-10085.59</v>
       </c>
       <c r="E980" t="n">
-        <v>-0.6328332454885426</v>
+        <v>-0.6328332454885425</v>
       </c>
     </row>
     <row r="981">
@@ -19194,7 +19194,7 @@
         <v>-10.55000000000001</v>
       </c>
       <c r="E981" t="n">
-        <v>-0.03109159495461511</v>
+        <v>-0.03109159495461515</v>
       </c>
     </row>
     <row r="982">
@@ -19285,7 +19285,7 @@
         <v>199.44</v>
       </c>
       <c r="E986" t="n">
-        <v>2.985628742514971</v>
+        <v>2.98562874251497</v>
       </c>
     </row>
     <row r="987">
@@ -19304,7 +19304,7 @@
         <v>809</v>
       </c>
       <c r="E987" t="n">
-        <v>0.0757490636704119</v>
+        <v>0.07574906367041198</v>
       </c>
     </row>
     <row r="988">
@@ -19357,7 +19357,7 @@
         <v>-0.01999999999998181</v>
       </c>
       <c r="E990" t="n">
-        <v>-4.534530449362695e-05</v>
+        <v>-4.534530449367843e-05</v>
       </c>
     </row>
     <row r="991">
@@ -19393,7 +19393,7 @@
         <v>0.01999999998952262</v>
       </c>
       <c r="E992" t="n">
-        <v>1.652237673344104e-07</v>
+        <v>1.652237674184895e-07</v>
       </c>
     </row>
     <row r="993">
@@ -19488,7 +19488,7 @@
         <v>1052.610000000001</v>
       </c>
       <c r="E997" t="n">
-        <v>0.08179747584992492</v>
+        <v>0.08179747584992494</v>
       </c>
     </row>
     <row r="998">
@@ -19524,7 +19524,7 @@
         <v>-2690.33</v>
       </c>
       <c r="E999" t="n">
-        <v>-0.8350186847430693</v>
+        <v>-0.8350186847430692</v>
       </c>
     </row>
     <row r="1000">
@@ -19562,7 +19562,7 @@
         <v>970.77</v>
       </c>
       <c r="E1001" t="n">
-        <v>-0.2826706034452636</v>
+        <v>0.2826706034452636</v>
       </c>
     </row>
     <row r="1002">
@@ -19600,7 +19600,7 @@
         <v>0.09000000000014552</v>
       </c>
       <c r="E1003" t="n">
-        <v>3.375000843686138e-06</v>
+        <v>3.375000843755668e-06</v>
       </c>
     </row>
     <row r="1004">
@@ -19619,7 +19619,7 @@
         <v>-486.6099999999997</v>
       </c>
       <c r="E1004" t="n">
-        <v>-0.186663035264242</v>
+        <v>-0.1866630352642419</v>
       </c>
     </row>
     <row r="1005">
@@ -19638,7 +19638,7 @@
         <v>234.48</v>
       </c>
       <c r="E1005" t="n">
-        <v>0.528108108108108</v>
+        <v>0.5281081081081082</v>
       </c>
     </row>
     <row r="1006">
@@ -19746,7 +19746,7 @@
         <v>498.8099999999999</v>
       </c>
       <c r="E1011" t="n">
-        <v>0.1515172686127395</v>
+        <v>0.1515172686127396</v>
       </c>
     </row>
     <row r="1012">
@@ -19820,7 +19820,7 @@
         <v>-1027.6</v>
       </c>
       <c r="E1015" t="n">
-        <v>-0.8098033807478624</v>
+        <v>-0.8098033807478625</v>
       </c>
     </row>
     <row r="1016">
@@ -19839,7 +19839,7 @@
         <v>-902.7599999999999</v>
       </c>
       <c r="E1016" t="n">
-        <v>-0.8562323349204242</v>
+        <v>-0.8562323349204241</v>
       </c>
     </row>
     <row r="1017">
@@ -19858,7 +19858,7 @@
         <v>227.27</v>
       </c>
       <c r="E1017" t="n">
-        <v>0.6532999885017823</v>
+        <v>0.6532999885017822</v>
       </c>
     </row>
     <row r="1018">
@@ -19896,7 +19896,7 @@
         <v>500</v>
       </c>
       <c r="E1019" t="n">
-        <v>0.01604278418027461</v>
+        <v>0.01604278418027469</v>
       </c>
     </row>
     <row r="1020">
@@ -19951,7 +19951,7 @@
         <v>112.25</v>
       </c>
       <c r="E1022" t="n">
-        <v>0.0520331157754208</v>
+        <v>0.0520331157754209</v>
       </c>
     </row>
     <row r="1023">
@@ -19989,7 +19989,7 @@
         <v>-68.85000000000014</v>
       </c>
       <c r="E1024" t="n">
-        <v>-0.03969718285496837</v>
+        <v>-0.03969718285496842</v>
       </c>
     </row>
     <row r="1025">
@@ -20046,7 +20046,7 @@
         <v>-41.2199999999998</v>
       </c>
       <c r="E1027" t="n">
-        <v>-0.01586263161135393</v>
+        <v>-0.0158626316113539</v>
       </c>
     </row>
     <row r="1028">
@@ -20101,7 +20101,7 @@
         <v>-106.6699999999996</v>
       </c>
       <c r="E1030" t="n">
-        <v>-0.02614505641028142</v>
+        <v>-0.02614505641028146</v>
       </c>
     </row>
     <row r="1031">
@@ -20137,7 +20137,7 @@
         <v>-375.0499999999993</v>
       </c>
       <c r="E1032" t="n">
-        <v>-0.03913836122917713</v>
+        <v>-0.03913836122917718</v>
       </c>
     </row>
     <row r="1033">
@@ -20209,7 +20209,7 @@
         <v>-54.89999999999964</v>
       </c>
       <c r="E1036" t="n">
-        <v>-0.008208449769221415</v>
+        <v>-0.0082084497692214</v>
       </c>
     </row>
     <row r="1037">
@@ -20317,7 +20317,7 @@
         <v>-2310.53</v>
       </c>
       <c r="E1042" t="n">
-        <v>-0.2922257944568249</v>
+        <v>-0.292225794456825</v>
       </c>
     </row>
     <row r="1043">
@@ -20406,7 +20406,7 @@
         <v>368.260000000002</v>
       </c>
       <c r="E1047" t="n">
-        <v>0.01453049525843264</v>
+        <v>0.01453049525843267</v>
       </c>
     </row>
     <row r="1048">
@@ -20480,7 +20480,7 @@
         <v>-27.54999999999995</v>
       </c>
       <c r="E1051" t="n">
-        <v>-0.08379718344131137</v>
+        <v>-0.08379718344131142</v>
       </c>
     </row>
     <row r="1052">
@@ -20590,7 +20590,7 @@
         <v>-600</v>
       </c>
       <c r="E1057" t="n">
-        <v>-0.05222386630690223</v>
+        <v>-0.05222386630690225</v>
       </c>
     </row>
     <row r="1058">
@@ -20679,7 +20679,7 @@
         <v>-0.01999999998952262</v>
       </c>
       <c r="E1062" t="n">
-        <v>-1.652237401339463e-07</v>
+        <v>-1.652237401196007e-07</v>
       </c>
     </row>
     <row r="1063">
@@ -20717,7 +20717,7 @@
         <v>24795.53</v>
       </c>
       <c r="E1064" t="n">
-        <v>-21.88156234280823</v>
+        <v>21.88156234280823</v>
       </c>
     </row>
     <row r="1065">
@@ -20736,7 +20736,7 @@
         <v>3835.33</v>
       </c>
       <c r="E1065" t="n">
-        <v>-6.772252926738827</v>
+        <v>6.772252926738827</v>
       </c>
     </row>
     <row r="1066">
@@ -20846,7 +20846,7 @@
         <v>376.5200000000004</v>
       </c>
       <c r="E1071" t="n">
-        <v>-0.1528388356450757</v>
+        <v>0.1528388356450757</v>
       </c>
     </row>
     <row r="1072">
@@ -20884,7 +20884,7 @@
         <v>-0.09000000000014552</v>
       </c>
       <c r="E1073" t="n">
-        <v>-3.374989453130972e-06</v>
+        <v>-3.374989453163416e-06</v>
       </c>
     </row>
     <row r="1074">
@@ -20903,7 +20903,7 @@
         <v>-8.840000000000146</v>
       </c>
       <c r="E1074" t="n">
-        <v>-0.004169260663685947</v>
+        <v>-0.004169260663685997</v>
       </c>
     </row>
     <row r="1075">
@@ -21030,7 +21030,7 @@
         <v>21.87000000000035</v>
       </c>
       <c r="E1081" t="n">
-        <v>0.005769063364733151</v>
+        <v>0.005769063364733098</v>
       </c>
     </row>
     <row r="1082">
@@ -21049,7 +21049,7 @@
         <v>712.9699999999999</v>
       </c>
       <c r="E1082" t="n">
-        <v>1.146125034160142</v>
+        <v>1.146125034160143</v>
       </c>
     </row>
     <row r="1083">
@@ -21102,7 +21102,7 @@
         <v>127.79</v>
       </c>
       <c r="E1085" t="n">
-        <v>0.5294800082867206</v>
+        <v>0.5294800082867205</v>
       </c>
     </row>
     <row r="1086">
@@ -21159,7 +21159,7 @@
         <v>2911.36</v>
       </c>
       <c r="E1088" t="n">
-        <v>91.17945505793924</v>
+        <v>91.17945505793925</v>
       </c>
     </row>
     <row r="1089">
@@ -21197,7 +21197,7 @@
         <v>3.129999999999995</v>
       </c>
       <c r="E1090" t="n">
-        <v>0.00746802824966597</v>
+        <v>0.007468028249665956</v>
       </c>
     </row>
     <row r="1091">
@@ -21328,7 +21328,7 @@
         <v>20.53999999999996</v>
       </c>
       <c r="E1097" t="n">
-        <v>0.008031783024548877</v>
+        <v>0.008031783024548931</v>
       </c>
     </row>
     <row r="1098">
@@ -21383,7 +21383,7 @@
         <v>-153.2200000000003</v>
       </c>
       <c r="E1100" t="n">
-        <v>-0.03856279226630033</v>
+        <v>-0.03856279226630028</v>
       </c>
     </row>
     <row r="1101">
@@ -21474,7 +21474,7 @@
         <v>1612.5</v>
       </c>
       <c r="E1105" t="n">
-        <v>0.337240795156281</v>
+        <v>0.3372407951562811</v>
       </c>
     </row>
     <row r="1106">
@@ -21582,7 +21582,7 @@
         <v>-0.08999999999650754</v>
       </c>
       <c r="E1111" t="n">
-        <v>-1.220337493723633e-06</v>
+        <v>-1.220337493778076e-06</v>
       </c>
     </row>
     <row r="1112">
@@ -21601,7 +21601,7 @@
         <v>476.8199999999997</v>
       </c>
       <c r="E1112" t="n">
-        <v>0.08520531152778799</v>
+        <v>0.0852053115277879</v>
       </c>
     </row>
     <row r="1113">
@@ -21620,7 +21620,7 @@
         <v>116.1300000000001</v>
       </c>
       <c r="E1113" t="n">
-        <v>0.04745617261248003</v>
+        <v>0.04745617261248013</v>
       </c>
     </row>
     <row r="1114">
@@ -21690,7 +21690,7 @@
         <v>2023.130000000001</v>
       </c>
       <c r="E1117" t="n">
-        <v>0.07868365989685833</v>
+        <v>0.07868365989685834</v>
       </c>
     </row>
     <row r="1118">
@@ -21726,7 +21726,7 @@
         <v>-0.3000000000000114</v>
       </c>
       <c r="E1119" t="n">
-        <v>-0.0006280355049406161</v>
+        <v>-0.0006280355049405698</v>
       </c>
     </row>
     <row r="1120">
@@ -21764,7 +21764,7 @@
         <v>-13.44000000000005</v>
       </c>
       <c r="E1121" t="n">
-        <v>-0.04461855122501845</v>
+        <v>-0.04461855122501843</v>
       </c>
     </row>
     <row r="1122">
@@ -21783,7 +21783,7 @@
         <v>268.3499999999999</v>
       </c>
       <c r="E1122" t="n">
-        <v>0.4524684696836849</v>
+        <v>0.452468469683685</v>
       </c>
     </row>
     <row r="1123">
@@ -21874,7 +21874,7 @@
         <v>300</v>
       </c>
       <c r="E1127" t="n">
-        <v>0.02755073927817064</v>
+        <v>0.02755073927817063</v>
       </c>
     </row>
     <row r="1128">
@@ -21963,7 +21963,7 @@
         <v>4706.199999999997</v>
       </c>
       <c r="E1132" t="n">
-        <v>0.0388788047316122</v>
+        <v>0.03887880473161213</v>
       </c>
     </row>
     <row r="1133">
@@ -22094,7 +22094,7 @@
         <v>2721.73</v>
       </c>
       <c r="E1139" t="n">
-        <v>1.80620221915481</v>
+        <v>1.806202219154809</v>
       </c>
     </row>
     <row r="1140">
@@ -22113,7 +22113,7 @@
         <v>167.2</v>
       </c>
       <c r="E1140" t="n">
-        <v>0.4773733047822986</v>
+        <v>0.4773733047822985</v>
       </c>
     </row>
     <row r="1141">
@@ -22132,7 +22132,7 @@
         <v>533.6999999999998</v>
       </c>
       <c r="E1141" t="n">
-        <v>-0.2557271477103388</v>
+        <v>0.2557271477103388</v>
       </c>
     </row>
     <row r="1142">
@@ -22168,7 +22168,7 @@
         <v>945.8400000000001</v>
       </c>
       <c r="E1143" t="n">
-        <v>0.03546900886725224</v>
+        <v>0.03546900886725222</v>
       </c>
     </row>
     <row r="1144">
@@ -22187,7 +22187,7 @@
         <v>75.92000000000007</v>
       </c>
       <c r="E1144" t="n">
-        <v>0.03595650361838376</v>
+        <v>0.0359565036183837</v>
       </c>
     </row>
     <row r="1145">
@@ -22206,7 +22206,7 @@
         <v>-1.299999999999955</v>
       </c>
       <c r="E1145" t="n">
-        <v>-0.002309099628767797</v>
+        <v>-0.002309099628767748</v>
       </c>
     </row>
     <row r="1146">
@@ -22335,7 +22335,7 @@
         <v>-215.73</v>
       </c>
       <c r="E1152" t="n">
-        <v>-0.1615906639501439</v>
+        <v>-0.1615906639501438</v>
       </c>
     </row>
     <row r="1153">
@@ -22428,7 +22428,7 @@
         <v>-22.66000000000003</v>
       </c>
       <c r="E1157" t="n">
-        <v>-0.06582999244669119</v>
+        <v>-0.06582999244669113</v>
       </c>
     </row>
     <row r="1158">
@@ -22447,7 +22447,7 @@
         <v>-2474.85</v>
       </c>
       <c r="E1158" t="n">
-        <v>-0.8408447689490333</v>
+        <v>-0.8408447689490332</v>
       </c>
     </row>
     <row r="1159">
@@ -22466,7 +22466,7 @@
         <v>979.1599999999999</v>
       </c>
       <c r="E1159" t="n">
-        <v>0.03092084861491551</v>
+        <v>0.03092084861491549</v>
       </c>
     </row>
     <row r="1160">
@@ -22485,7 +22485,7 @@
         <v>83.69999999999999</v>
       </c>
       <c r="E1160" t="n">
-        <v>0.1982238010657194</v>
+        <v>0.1982238010657193</v>
       </c>
     </row>
     <row r="1161">
@@ -22521,7 +22521,7 @@
         <v>74.89999999999964</v>
       </c>
       <c r="E1162" t="n">
-        <v>0.0330024278154506</v>
+        <v>0.03300242781545061</v>
       </c>
     </row>
     <row r="1163">
@@ -22559,7 +22559,7 @@
         <v>-32.02999999999997</v>
       </c>
       <c r="E1164" t="n">
-        <v>-0.02594341532953726</v>
+        <v>-0.02594341532953724</v>
       </c>
     </row>
     <row r="1165">
@@ -22616,7 +22616,7 @@
         <v>19.59999999999991</v>
       </c>
       <c r="E1167" t="n">
-        <v>0.007603146771765878</v>
+        <v>0.007603146771765911</v>
       </c>
     </row>
     <row r="1168">
@@ -22669,7 +22669,7 @@
         <v>-208.1500000000001</v>
       </c>
       <c r="E1170" t="n">
-        <v>-0.05448895823080391</v>
+        <v>-0.05448895823080389</v>
       </c>
     </row>
     <row r="1171">
@@ -22705,7 +22705,7 @@
         <v>370.2199999999993</v>
       </c>
       <c r="E1172" t="n">
-        <v>0.04020800163342964</v>
+        <v>0.04020800163342963</v>
       </c>
     </row>
     <row r="1173">
@@ -22758,7 +22758,7 @@
         <v>-1612.5</v>
       </c>
       <c r="E1175" t="n">
-        <v>-0.2521915248007882</v>
+        <v>-0.2521915248007883</v>
       </c>
     </row>
     <row r="1176">
@@ -22866,7 +22866,7 @@
         <v>3262.5</v>
       </c>
       <c r="E1181" t="n">
-        <v>0.04423728813559324</v>
+        <v>0.04423728813559322</v>
       </c>
     </row>
     <row r="1182">
@@ -22885,7 +22885,7 @@
         <v>35.90999999999985</v>
       </c>
       <c r="E1182" t="n">
-        <v>0.005913106480376129</v>
+        <v>0.00591310648037607</v>
       </c>
     </row>
     <row r="1183">
@@ -22904,7 +22904,7 @@
         <v>-121.1399999999999</v>
       </c>
       <c r="E1183" t="n">
-        <v>-0.04726068281036033</v>
+        <v>-0.04726068281036032</v>
       </c>
     </row>
     <row r="1184">
@@ -22974,7 +22974,7 @@
         <v>3012.779999999999</v>
       </c>
       <c r="E1187" t="n">
-        <v>0.1086260736757052</v>
+        <v>0.1086260736757053</v>
       </c>
     </row>
     <row r="1188">
@@ -23048,7 +23048,7 @@
         <v>-1.899999999999977</v>
       </c>
       <c r="E1191" t="n">
-        <v>-0.006602265619570447</v>
+        <v>-0.006602265619570427</v>
       </c>
     </row>
     <row r="1192">
@@ -23067,7 +23067,7 @@
         <v>345.14</v>
       </c>
       <c r="E1192" t="n">
-        <v>0.4006593687240982</v>
+        <v>0.4006593687240983</v>
       </c>
     </row>
     <row r="1193">
@@ -23160,7 +23160,7 @@
         <v>-300</v>
       </c>
       <c r="E1197" t="n">
-        <v>-0.02681204754669764</v>
+        <v>-0.02681204754669765</v>
       </c>
     </row>
     <row r="1198">
@@ -23213,7 +23213,7 @@
         <v>0.009999999999990905</v>
       </c>
       <c r="E1200" t="n">
-        <v>2.267368039188256e-05</v>
+        <v>2.267368039178057e-05</v>
       </c>
     </row>
     <row r="1201">
@@ -23325,7 +23325,7 @@
         <v>-176</v>
       </c>
       <c r="E1206" t="n">
-        <v>-0.5419553502694381</v>
+        <v>-0.541955350269438</v>
       </c>
     </row>
     <row r="1207">
@@ -23344,7 +23344,7 @@
         <v>678.6499999999996</v>
       </c>
       <c r="E1207" t="n">
-        <v>0.04475293071851971</v>
+        <v>0.04475293071851977</v>
       </c>
     </row>
     <row r="1208">
@@ -23380,7 +23380,7 @@
         <v>1772.47</v>
       </c>
       <c r="E1209" t="n">
-        <v>0.4191613792712028</v>
+        <v>0.4191613792712027</v>
       </c>
     </row>
     <row r="1210">
@@ -23418,7 +23418,7 @@
         <v>223.6499999999999</v>
       </c>
       <c r="E1211" t="n">
-        <v>-0.1439847034359327</v>
+        <v>0.1439847034359327</v>
       </c>
     </row>
     <row r="1212">
@@ -23494,7 +23494,7 @@
         <v>29.7299999999999</v>
       </c>
       <c r="E1215" t="n">
-        <v>0.05292955188805193</v>
+        <v>0.05292955188805196</v>
       </c>
     </row>
     <row r="1216">
@@ -23566,7 +23566,7 @@
         <v>343.9300000000003</v>
       </c>
       <c r="E1219" t="n">
-        <v>0.07774871654598847</v>
+        <v>0.07774871654598853</v>
       </c>
     </row>
     <row r="1220">
@@ -23642,7 +23642,7 @@
         <v>-8394.630000000001</v>
       </c>
       <c r="E1223" t="n">
-        <v>-0.6761639876666119</v>
+        <v>-0.676163987666612</v>
       </c>
     </row>
     <row r="1224">
@@ -23678,7 +23678,7 @@
         <v>-36.81</v>
       </c>
       <c r="E1225" t="n">
-        <v>-0.2269560392132685</v>
+        <v>-0.2269560392132684</v>
       </c>
     </row>
     <row r="1226">
@@ -23697,7 +23697,7 @@
         <v>-68.44</v>
       </c>
       <c r="E1226" t="n">
-        <v>-0.1406118381854417</v>
+        <v>-0.1406118381854416</v>
       </c>
     </row>
     <row r="1227">
@@ -23735,7 +23735,7 @@
         <v>-318.19</v>
       </c>
       <c r="E1228" t="n">
-        <v>-0.6792545470070874</v>
+        <v>-0.6792545470070873</v>
       </c>
     </row>
     <row r="1229">
@@ -23773,7 +23773,7 @@
         <v>14.55000000000001</v>
       </c>
       <c r="E1230" t="n">
-        <v>0.02875778238956417</v>
+        <v>0.02875778238956421</v>
       </c>
     </row>
     <row r="1231">
@@ -23847,7 +23847,7 @@
         <v>100.5500000000002</v>
       </c>
       <c r="E1234" t="n">
-        <v>0.08361190107934613</v>
+        <v>0.08361190107934623</v>
       </c>
     </row>
     <row r="1235">
@@ -23904,7 +23904,7 @@
         <v>-9.800000000000182</v>
       </c>
       <c r="E1237" t="n">
-        <v>-0.003772887567950578</v>
+        <v>-0.003772887567950545</v>
       </c>
     </row>
     <row r="1238">
@@ -23959,7 +23959,7 @@
         <v>321.2800000000002</v>
       </c>
       <c r="E1240" t="n">
-        <v>0.0889506601806811</v>
+        <v>0.08895066018068108</v>
       </c>
     </row>
     <row r="1241">
@@ -23995,7 +23995,7 @@
         <v>-7.659999999999854</v>
       </c>
       <c r="E1242" t="n">
-        <v>-0.000799762785763769</v>
+        <v>-0.0007997627857637896</v>
       </c>
     </row>
     <row r="1243">
@@ -24048,7 +24048,7 @@
         <v>-159.1999999999998</v>
       </c>
       <c r="E1245" t="n">
-        <v>-0.03329533927992556</v>
+        <v>-0.03329533927992551</v>
       </c>
     </row>
     <row r="1246">
@@ -24086,7 +24086,7 @@
         <v>1574.08</v>
       </c>
       <c r="E1247" t="n">
-        <v>0.1040546186268132</v>
+        <v>0.1040546186268133</v>
       </c>
     </row>
     <row r="1248">
@@ -24156,7 +24156,7 @@
         <v>-2863.630000000005</v>
       </c>
       <c r="E1251" t="n">
-        <v>-0.03718396364226595</v>
+        <v>-0.03718396364226593</v>
       </c>
     </row>
     <row r="1252">
@@ -24175,7 +24175,7 @@
         <v>731.2800000000007</v>
       </c>
       <c r="E1252" t="n">
-        <v>0.1197080961095851</v>
+        <v>0.1197080961095852</v>
       </c>
     </row>
     <row r="1253">
@@ -24194,7 +24194,7 @@
         <v>432.71</v>
       </c>
       <c r="E1253" t="n">
-        <v>0.177188391910208</v>
+        <v>0.1771883919102081</v>
       </c>
     </row>
     <row r="1254">
@@ -24264,7 +24264,7 @@
         <v>1657.419999999998</v>
       </c>
       <c r="E1257" t="n">
-        <v>0.05390315047006133</v>
+        <v>0.05390315047006135</v>
       </c>
     </row>
     <row r="1258">
@@ -24319,7 +24319,7 @@
         <v>2973.25</v>
       </c>
       <c r="E1260" t="n">
-        <v>7.411816028916865</v>
+        <v>7.411816028916864</v>
       </c>
     </row>
     <row r="1261">
@@ -24338,7 +24338,7 @@
         <v>15.88</v>
       </c>
       <c r="E1261" t="n">
-        <v>0.05554778228627399</v>
+        <v>0.05554778228627395</v>
       </c>
     </row>
   </sheetData>

</xml_diff>